<commit_message>
Set Python version to 3.12.10
</commit_message>
<xml_diff>
--- a/predictions_log.xlsx
+++ b/predictions_log.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -510,6 +510,99 @@
       <c r="S1" t="inlineStr">
         <is>
           <t>Feedback</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>2026-02-22 10:23:29</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>34</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>MALE</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>STRAW</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>SLIGHTLY HAZY</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>NEGATIVE</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>NEGATIVE</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>OCCASIONAL</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>RARE</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>NEGATIVE</t>
+        </is>
+      </c>
+      <c r="R2" t="n">
+        <v>99.7</v>
+      </c>
+      <c r="S2" t="inlineStr">
+        <is>
+          <t>Not provided</t>
         </is>
       </c>
     </row>

</xml_diff>